<commit_message>
Update analysis script and figures
</commit_message>
<xml_diff>
--- a/CNC_UK_data_overview.xlsx
+++ b/CNC_UK_data_overview.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hullacuk-my.sharepoint.com/personal/b_hodgson-2022_hull_ac_uk/Documents/Aa. Dissertation/Data and Analysis/GitHub folder/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="173" documentId="11_40EA3C77D094CE56413DCE42115AF69F046E0E85" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1A6975A4-C25D-4925-B7C9-1D2911E618FD}"/>
+  <xr:revisionPtr revIDLastSave="401" documentId="11_40EA3C77D094CE56413DCE42115AF69F046E0E85" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2D79F7A7-4A78-48D8-9342-68C5DD9DF06F}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Participation_by_year" sheetId="5" r:id="rId1"/>
@@ -18,12 +18,25 @@
     <sheet name="Included_project_details" sheetId="2" r:id="rId3"/>
     <sheet name="Data_sources" sheetId="3" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="644" uniqueCount="323">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="649" uniqueCount="326">
   <si>
     <t>city</t>
   </si>
@@ -607,9 +620,6 @@
     <t>Year threshold not met</t>
   </si>
   <si>
-    <t>Urban cover and year thresholds not met</t>
-  </si>
-  <si>
     <t>Dundee City</t>
   </si>
   <si>
@@ -992,6 +1002,18 @@
   </si>
   <si>
     <t>City Nature Challenge 2025: Warwickshire, Coventry and Solihull · iNaturalist United Kingdom</t>
+  </si>
+  <si>
+    <t>Participation threshold not met</t>
+  </si>
+  <si>
+    <t>Urban cover and participation thresholds not met</t>
+  </si>
+  <si>
+    <t>Outside England</t>
+  </si>
+  <si>
+    <t>Unfeasible, excluded following feasibility screening</t>
   </si>
 </sst>
 </file>
@@ -1079,7 +1101,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1095,11 +1117,7 @@
     </xf>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1116,10 +1134,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1443,11 +1457,11 @@
       <c r="G2" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="H2" s="10" t="s">
+      <c r="H2" s="9" t="s">
+        <v>200</v>
+      </c>
+      <c r="I2" s="9" t="s">
         <v>201</v>
-      </c>
-      <c r="I2" s="10" t="s">
-        <v>202</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -1460,23 +1474,23 @@
       <c r="C3" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="D3" s="10" t="s">
+      <c r="D3" s="9" t="s">
+        <v>202</v>
+      </c>
+      <c r="E3" s="9" t="s">
         <v>203</v>
       </c>
-      <c r="E3" s="10" t="s">
+      <c r="F3" s="9" t="s">
         <v>204</v>
       </c>
-      <c r="F3" s="10" t="s">
+      <c r="G3" s="9" t="s">
         <v>205</v>
       </c>
-      <c r="G3" s="10" t="s">
+      <c r="H3" s="9" t="s">
         <v>206</v>
       </c>
-      <c r="H3" s="10" t="s">
+      <c r="I3" s="9" t="s">
         <v>207</v>
-      </c>
-      <c r="I3" s="10" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -1489,57 +1503,57 @@
       <c r="C4" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="D4" s="10" t="s">
+      <c r="D4" s="9" t="s">
+        <v>208</v>
+      </c>
+      <c r="E4" s="9" t="s">
         <v>209</v>
       </c>
-      <c r="E4" s="10" t="s">
+      <c r="F4" s="9" t="s">
         <v>210</v>
       </c>
-      <c r="F4" s="10" t="s">
+      <c r="G4" s="9" t="s">
         <v>211</v>
       </c>
-      <c r="G4" s="10" t="s">
+      <c r="H4" s="9" t="s">
         <v>212</v>
       </c>
-      <c r="H4" s="10" t="s">
+      <c r="I4" s="9" t="s">
         <v>213</v>
-      </c>
-      <c r="I4" s="10" t="s">
-        <v>214</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="B5" s="9" t="s">
         <v>261</v>
       </c>
-      <c r="B5" s="10" t="s">
+      <c r="C5" s="9" t="s">
         <v>262</v>
       </c>
-      <c r="C5" s="10" t="s">
+      <c r="D5" s="9" t="s">
         <v>263</v>
       </c>
-      <c r="D5" s="10" t="s">
+      <c r="E5" s="9" t="s">
         <v>264</v>
       </c>
-      <c r="E5" s="10" t="s">
+      <c r="F5" s="9" t="s">
         <v>265</v>
       </c>
-      <c r="F5" s="10" t="s">
+      <c r="G5" s="9" t="s">
         <v>266</v>
       </c>
-      <c r="G5" s="10" t="s">
+      <c r="H5" s="9" t="s">
         <v>267</v>
       </c>
-      <c r="H5" s="10" t="s">
-        <v>268</v>
-      </c>
-      <c r="I5" s="10" t="s">
-        <v>260</v>
+      <c r="I5" s="9" t="s">
+        <v>259</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>187</v>
@@ -1550,49 +1564,49 @@
       <c r="D6" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="E6" s="10" t="s">
+      <c r="E6" s="9" t="s">
+        <v>222</v>
+      </c>
+      <c r="F6" s="9" t="s">
         <v>223</v>
       </c>
-      <c r="F6" s="10" t="s">
+      <c r="G6" s="9" t="s">
         <v>224</v>
       </c>
-      <c r="G6" s="10" t="s">
+      <c r="H6" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="I6" s="9" t="s">
         <v>225</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>187</v>
-      </c>
-      <c r="I6" s="10" t="s">
-        <v>226</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="G7" s="9" t="s">
+        <v>226</v>
+      </c>
+      <c r="H7" s="9" t="s">
         <v>228</v>
       </c>
-      <c r="B7" s="1" t="s">
-        <v>187</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>187</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>187</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>187</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>187</v>
-      </c>
-      <c r="G7" s="10" t="s">
-        <v>227</v>
-      </c>
-      <c r="H7" s="10" t="s">
-        <v>229</v>
-      </c>
-      <c r="I7" s="10" t="s">
-        <v>231</v>
+      <c r="I7" s="9" t="s">
+        <v>230</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
@@ -1620,8 +1634,8 @@
       <c r="H8" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="I8" s="10" t="s">
-        <v>232</v>
+      <c r="I8" s="9" t="s">
+        <v>231</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
@@ -1637,17 +1651,17 @@
       <c r="D9" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="E9" s="10" t="s">
+      <c r="E9" s="9" t="s">
+        <v>232</v>
+      </c>
+      <c r="F9" s="9" t="s">
         <v>233</v>
       </c>
-      <c r="F9" s="10" t="s">
+      <c r="G9" s="9" t="s">
         <v>234</v>
       </c>
-      <c r="G9" s="10" t="s">
+      <c r="H9" s="9" t="s">
         <v>235</v>
-      </c>
-      <c r="H9" s="10" t="s">
-        <v>236</v>
       </c>
       <c r="I9" s="1" t="s">
         <v>187</v>
@@ -1672,8 +1686,8 @@
       <c r="F10" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="G10" s="10" t="s">
-        <v>237</v>
+      <c r="G10" s="9" t="s">
+        <v>236</v>
       </c>
       <c r="H10" s="1" t="s">
         <v>187</v>
@@ -1701,14 +1715,14 @@
       <c r="F11" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="G11" s="10" t="s">
+      <c r="G11" s="9" t="s">
+        <v>237</v>
+      </c>
+      <c r="H11" s="9" t="s">
         <v>238</v>
       </c>
-      <c r="H11" s="10" t="s">
+      <c r="I11" s="9" t="s">
         <v>239</v>
-      </c>
-      <c r="I11" s="10" t="s">
-        <v>240</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
@@ -1736,8 +1750,8 @@
       <c r="H12" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="I12" s="10" t="s">
-        <v>241</v>
+      <c r="I12" s="9" t="s">
+        <v>240</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
@@ -1753,17 +1767,17 @@
       <c r="D13" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="E13" s="10" t="s">
+      <c r="E13" s="9" t="s">
+        <v>241</v>
+      </c>
+      <c r="F13" s="9" t="s">
         <v>242</v>
       </c>
-      <c r="F13" s="10" t="s">
+      <c r="G13" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="G13" s="10" t="s">
+      <c r="H13" s="9" t="s">
         <v>244</v>
-      </c>
-      <c r="H13" s="10" t="s">
-        <v>245</v>
       </c>
       <c r="I13" s="1" t="s">
         <v>187</v>
@@ -1791,11 +1805,11 @@
       <c r="G14" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="H14" s="10" t="s">
+      <c r="H14" s="9" t="s">
+        <v>245</v>
+      </c>
+      <c r="I14" s="9" t="s">
         <v>246</v>
-      </c>
-      <c r="I14" s="10" t="s">
-        <v>247</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
@@ -1811,20 +1825,20 @@
       <c r="D15" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="E15" s="10" t="s">
+      <c r="E15" s="9" t="s">
+        <v>247</v>
+      </c>
+      <c r="F15" s="9" t="s">
         <v>248</v>
       </c>
-      <c r="F15" s="10" t="s">
+      <c r="G15" s="9" t="s">
         <v>249</v>
       </c>
-      <c r="G15" s="10" t="s">
+      <c r="H15" s="9" t="s">
         <v>250</v>
       </c>
-      <c r="H15" s="10" t="s">
+      <c r="I15" s="9" t="s">
         <v>251</v>
-      </c>
-      <c r="I15" s="10" t="s">
-        <v>252</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
@@ -1832,55 +1846,55 @@
         <v>43</v>
       </c>
       <c r="B16" s="1"/>
-      <c r="C16" s="10" t="s">
+      <c r="C16" s="9" t="s">
+        <v>252</v>
+      </c>
+      <c r="D16" s="9" t="s">
         <v>253</v>
       </c>
-      <c r="D16" s="10" t="s">
+      <c r="E16" s="9" t="s">
         <v>254</v>
       </c>
-      <c r="E16" s="10" t="s">
+      <c r="F16" s="9" t="s">
         <v>255</v>
       </c>
-      <c r="F16" s="10" t="s">
+      <c r="G16" s="9" t="s">
         <v>256</v>
       </c>
-      <c r="G16" s="10" t="s">
+      <c r="H16" s="9" t="s">
         <v>257</v>
       </c>
-      <c r="H16" s="10" t="s">
+      <c r="I16" s="9" t="s">
         <v>258</v>
-      </c>
-      <c r="I16" s="10" t="s">
-        <v>259</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B17" s="10" t="s">
+      <c r="B17" s="9" t="s">
+        <v>214</v>
+      </c>
+      <c r="C17" s="9" t="s">
         <v>215</v>
       </c>
-      <c r="C17" s="10" t="s">
+      <c r="D17" s="9" t="s">
         <v>216</v>
       </c>
-      <c r="D17" s="10" t="s">
+      <c r="E17" s="9" t="s">
         <v>217</v>
       </c>
-      <c r="E17" s="10" t="s">
+      <c r="F17" s="9" t="s">
         <v>218</v>
       </c>
-      <c r="F17" s="10" t="s">
+      <c r="G17" s="9" t="s">
         <v>219</v>
       </c>
-      <c r="G17" s="10" t="s">
+      <c r="H17" s="9" t="s">
         <v>220</v>
       </c>
-      <c r="H17" s="10" t="s">
+      <c r="I17" s="9" t="s">
         <v>221</v>
-      </c>
-      <c r="I17" s="10" t="s">
-        <v>222</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
@@ -1890,26 +1904,26 @@
       <c r="B18" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="C18" s="10" t="s">
+      <c r="C18" s="9" t="s">
+        <v>268</v>
+      </c>
+      <c r="D18" s="9" t="s">
         <v>269</v>
       </c>
-      <c r="D18" s="10" t="s">
+      <c r="E18" s="9" t="s">
         <v>270</v>
       </c>
-      <c r="E18" s="10" t="s">
+      <c r="F18" s="9" t="s">
         <v>271</v>
       </c>
-      <c r="F18" s="10" t="s">
+      <c r="G18" s="9" t="s">
         <v>272</v>
       </c>
-      <c r="G18" s="10" t="s">
+      <c r="H18" s="9" t="s">
         <v>273</v>
       </c>
-      <c r="H18" s="10" t="s">
+      <c r="I18" s="9" t="s">
         <v>274</v>
-      </c>
-      <c r="I18" s="10" t="s">
-        <v>275</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
@@ -1934,11 +1948,11 @@
       <c r="G19" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="H19" s="10" t="s">
-        <v>277</v>
-      </c>
-      <c r="I19" s="10" t="s">
+      <c r="H19" s="9" t="s">
         <v>276</v>
+      </c>
+      <c r="I19" s="9" t="s">
+        <v>275</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
@@ -1966,8 +1980,8 @@
       <c r="H20" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="I20" s="10" t="s">
-        <v>278</v>
+      <c r="I20" s="9" t="s">
+        <v>277</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
@@ -1995,8 +2009,8 @@
       <c r="H21" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="I21" s="10" t="s">
-        <v>279</v>
+      <c r="I21" s="9" t="s">
+        <v>278</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
@@ -2018,14 +2032,14 @@
       <c r="F22" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="G22" s="10" t="s">
-        <v>282</v>
-      </c>
-      <c r="H22" s="10" t="s">
+      <c r="G22" s="9" t="s">
         <v>281</v>
       </c>
-      <c r="I22" s="10" t="s">
+      <c r="H22" s="9" t="s">
         <v>280</v>
+      </c>
+      <c r="I22" s="9" t="s">
+        <v>279</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
@@ -2038,23 +2052,23 @@
       <c r="C23" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="D23" s="10" t="s">
+      <c r="D23" s="9" t="s">
+        <v>282</v>
+      </c>
+      <c r="E23" s="9" t="s">
         <v>283</v>
       </c>
-      <c r="E23" s="10" t="s">
+      <c r="F23" s="9" t="s">
         <v>284</v>
       </c>
-      <c r="F23" s="10" t="s">
+      <c r="G23" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="H23" s="9" t="s">
         <v>285</v>
       </c>
-      <c r="G23" s="1" t="s">
-        <v>187</v>
-      </c>
-      <c r="H23" s="10" t="s">
+      <c r="I23" s="9" t="s">
         <v>286</v>
-      </c>
-      <c r="I23" s="10" t="s">
-        <v>287</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
@@ -2064,8 +2078,8 @@
       <c r="B24" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="C24" s="10" t="s">
-        <v>288</v>
+      <c r="C24" s="9" t="s">
+        <v>287</v>
       </c>
       <c r="D24" s="1" t="s">
         <v>187</v>
@@ -2093,26 +2107,26 @@
       <c r="B25" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="C25" s="10" t="s">
+      <c r="C25" s="9" t="s">
+        <v>288</v>
+      </c>
+      <c r="D25" s="9" t="s">
         <v>289</v>
       </c>
-      <c r="D25" s="10" t="s">
+      <c r="E25" s="9" t="s">
         <v>290</v>
       </c>
-      <c r="E25" s="10" t="s">
+      <c r="F25" s="9" t="s">
         <v>291</v>
       </c>
-      <c r="F25" s="10" t="s">
+      <c r="G25" s="9" t="s">
         <v>292</v>
       </c>
-      <c r="G25" s="10" t="s">
+      <c r="H25" s="9" t="s">
         <v>293</v>
       </c>
-      <c r="H25" s="10" t="s">
+      <c r="I25" s="9" t="s">
         <v>294</v>
-      </c>
-      <c r="I25" s="10" t="s">
-        <v>295</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
@@ -2122,26 +2136,26 @@
       <c r="B26" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="C26" s="10" t="s">
-        <v>302</v>
-      </c>
-      <c r="D26" s="10" t="s">
+      <c r="C26" s="9" t="s">
+        <v>301</v>
+      </c>
+      <c r="D26" s="9" t="s">
+        <v>296</v>
+      </c>
+      <c r="E26" s="9" t="s">
         <v>297</v>
       </c>
-      <c r="E26" s="10" t="s">
+      <c r="F26" s="9" t="s">
         <v>298</v>
       </c>
-      <c r="F26" s="10" t="s">
+      <c r="G26" s="9" t="s">
         <v>299</v>
       </c>
-      <c r="G26" s="10" t="s">
+      <c r="H26" s="9" t="s">
         <v>300</v>
       </c>
-      <c r="H26" s="10" t="s">
-        <v>301</v>
-      </c>
-      <c r="I26" s="10" t="s">
-        <v>296</v>
+      <c r="I26" s="9" t="s">
+        <v>295</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
@@ -2154,23 +2168,23 @@
       <c r="C27" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="D27" s="10" t="s">
+      <c r="D27" s="9" t="s">
+        <v>302</v>
+      </c>
+      <c r="E27" s="9" t="s">
         <v>303</v>
       </c>
-      <c r="E27" s="10" t="s">
+      <c r="F27" s="9" t="s">
         <v>304</v>
       </c>
-      <c r="F27" s="10" t="s">
+      <c r="G27" s="9" t="s">
         <v>305</v>
       </c>
-      <c r="G27" s="10" t="s">
+      <c r="H27" s="9" t="s">
         <v>306</v>
       </c>
-      <c r="H27" s="10" t="s">
+      <c r="I27" s="9" t="s">
         <v>307</v>
-      </c>
-      <c r="I27" s="10" t="s">
-        <v>308</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
@@ -2192,22 +2206,22 @@
       <c r="F28" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="G28" s="10" t="s">
+      <c r="G28" s="9" t="s">
+        <v>308</v>
+      </c>
+      <c r="H28" s="9" t="s">
         <v>309</v>
       </c>
-      <c r="H28" s="10" t="s">
+      <c r="I28" s="9" t="s">
         <v>310</v>
-      </c>
-      <c r="I28" s="10" t="s">
-        <v>311</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>174</v>
       </c>
-      <c r="B29" s="10" t="s">
-        <v>314</v>
+      <c r="B29" s="9" t="s">
+        <v>313</v>
       </c>
       <c r="C29" s="1" t="s">
         <v>187</v>
@@ -2253,11 +2267,11 @@
       <c r="G30" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="H30" s="10" t="s">
+      <c r="H30" s="9" t="s">
+        <v>311</v>
+      </c>
+      <c r="I30" s="9" t="s">
         <v>312</v>
-      </c>
-      <c r="I30" s="10" t="s">
-        <v>313</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
@@ -2279,11 +2293,11 @@
       <c r="F31" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="G31" s="10" t="s">
+      <c r="G31" s="9" t="s">
+        <v>314</v>
+      </c>
+      <c r="H31" s="9" t="s">
         <v>315</v>
-      </c>
-      <c r="H31" s="10" t="s">
-        <v>316</v>
       </c>
       <c r="I31" s="1" t="s">
         <v>187</v>
@@ -2308,14 +2322,14 @@
       <c r="F32" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="G32" s="10" t="s">
+      <c r="G32" s="9" t="s">
+        <v>316</v>
+      </c>
+      <c r="H32" s="9" t="s">
         <v>317</v>
       </c>
-      <c r="H32" s="10" t="s">
+      <c r="I32" s="9" t="s">
         <v>318</v>
-      </c>
-      <c r="I32" s="10" t="s">
-        <v>319</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
@@ -2337,14 +2351,14 @@
       <c r="F33" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="G33" s="10" t="s">
+      <c r="G33" s="9" t="s">
+        <v>319</v>
+      </c>
+      <c r="H33" s="9" t="s">
         <v>320</v>
       </c>
-      <c r="H33" s="10" t="s">
+      <c r="I33" s="9" t="s">
         <v>321</v>
-      </c>
-      <c r="I33" s="10" t="s">
-        <v>322</v>
       </c>
     </row>
   </sheetData>
@@ -2516,10 +2530,10 @@
         <v>4</v>
       </c>
       <c r="H1" t="s">
+        <v>198</v>
+      </c>
+      <c r="I1" t="s">
         <v>199</v>
-      </c>
-      <c r="I1" t="s">
-        <v>200</v>
       </c>
       <c r="J1" t="s">
         <v>21</v>
@@ -2541,7 +2555,7 @@
       <c r="B2" t="s">
         <v>36</v>
       </c>
-      <c r="C2" s="9" t="s">
+      <c r="C2" t="s">
         <v>182</v>
       </c>
       <c r="D2">
@@ -2566,7 +2580,7 @@
         <v>160</v>
       </c>
       <c r="L2" t="s">
-        <v>194</v>
+        <v>323</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
@@ -2576,7 +2590,7 @@
       <c r="B3" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="C3" t="s">
         <v>172</v>
       </c>
       <c r="D3">
@@ -2611,7 +2625,7 @@
       <c r="B4" t="s">
         <v>188</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="C4" t="s">
         <v>172</v>
       </c>
       <c r="D4">
@@ -2641,12 +2655,12 @@
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B5" t="s">
         <v>189</v>
       </c>
-      <c r="C5" s="9" t="s">
+      <c r="C5" t="s">
         <v>26</v>
       </c>
       <c r="D5">
@@ -2676,12 +2690,12 @@
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B6" t="s">
         <v>41</v>
       </c>
-      <c r="C6" s="9" t="s">
+      <c r="C6" t="s">
         <v>186</v>
       </c>
       <c r="D6">
@@ -2705,15 +2719,18 @@
       <c r="K6" t="s">
         <v>160</v>
       </c>
+      <c r="L6" t="s">
+        <v>324</v>
+      </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A7" s="11" t="s">
-        <v>228</v>
+      <c r="A7" t="s">
+        <v>227</v>
       </c>
       <c r="B7" t="s">
         <v>168</v>
       </c>
-      <c r="C7" s="9" t="s">
+      <c r="C7" t="s">
         <v>171</v>
       </c>
       <c r="D7">
@@ -2743,12 +2760,12 @@
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B8" t="s">
-        <v>197</v>
-      </c>
-      <c r="C8" s="9">
+        <v>196</v>
+      </c>
+      <c r="C8">
         <v>2025</v>
       </c>
       <c r="D8">
@@ -2757,8 +2774,8 @@
       <c r="E8">
         <v>1</v>
       </c>
-      <c r="H8" s="9" t="s">
-        <v>198</v>
+      <c r="H8" t="s">
+        <v>197</v>
       </c>
       <c r="I8">
         <v>-2.2124999999999999</v>
@@ -2767,7 +2784,7 @@
         <v>160</v>
       </c>
       <c r="L8" t="s">
-        <v>193</v>
+        <v>322</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
@@ -2777,7 +2794,7 @@
       <c r="B9" t="s">
         <v>40</v>
       </c>
-      <c r="C9" s="9" t="s">
+      <c r="C9" t="s">
         <v>181</v>
       </c>
       <c r="D9">
@@ -2800,6 +2817,9 @@
       </c>
       <c r="K9" t="s">
         <v>160</v>
+      </c>
+      <c r="L9" t="s">
+        <v>325</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
@@ -2809,7 +2829,7 @@
       <c r="B10" t="s">
         <v>176</v>
       </c>
-      <c r="C10" s="9">
+      <c r="C10">
         <v>2023</v>
       </c>
       <c r="D10">
@@ -2833,12 +2853,12 @@
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B11" t="s">
         <v>38</v>
       </c>
-      <c r="C11" s="9" t="s">
+      <c r="C11" t="s">
         <v>171</v>
       </c>
       <c r="D11">
@@ -2861,6 +2881,9 @@
       </c>
       <c r="K11" t="s">
         <v>160</v>
+      </c>
+      <c r="L11" t="s">
+        <v>324</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
@@ -2870,7 +2893,7 @@
       <c r="B12" t="s">
         <v>178</v>
       </c>
-      <c r="C12" s="9">
+      <c r="C12">
         <v>2025</v>
       </c>
       <c r="D12">
@@ -2889,7 +2912,7 @@
         <v>160</v>
       </c>
       <c r="L12" t="s">
-        <v>193</v>
+        <v>322</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
@@ -2899,7 +2922,7 @@
       <c r="B13" t="s">
         <v>39</v>
       </c>
-      <c r="C13" s="9" t="s">
+      <c r="C13" t="s">
         <v>181</v>
       </c>
       <c r="D13">
@@ -2934,7 +2957,7 @@
       <c r="B14" t="s">
         <v>167</v>
       </c>
-      <c r="C14" s="9" t="s">
+      <c r="C14" t="s">
         <v>182</v>
       </c>
       <c r="D14">
@@ -2953,7 +2976,7 @@
         <v>160</v>
       </c>
       <c r="L14" t="s">
-        <v>193</v>
+        <v>322</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
@@ -2963,7 +2986,7 @@
       <c r="B15" t="s">
         <v>166</v>
       </c>
-      <c r="C15" s="9" t="s">
+      <c r="C15" t="s">
         <v>183</v>
       </c>
       <c r="D15">
@@ -2998,7 +3021,7 @@
       <c r="B16" t="s">
         <v>165</v>
       </c>
-      <c r="C16" s="9" t="s">
+      <c r="C16" t="s">
         <v>173</v>
       </c>
       <c r="D16">
@@ -3033,7 +3056,7 @@
       <c r="B17" t="s">
         <v>6</v>
       </c>
-      <c r="C17" s="9" t="s">
+      <c r="C17" t="s">
         <v>26</v>
       </c>
       <c r="D17">
@@ -3068,7 +3091,7 @@
       <c r="B18" t="s">
         <v>8</v>
       </c>
-      <c r="C18" s="9" t="s">
+      <c r="C18" t="s">
         <v>173</v>
       </c>
       <c r="D18">
@@ -3097,13 +3120,13 @@
       </c>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A19" s="11" t="s">
+      <c r="A19" t="s">
         <v>190</v>
       </c>
       <c r="B19" t="s">
         <v>190</v>
       </c>
-      <c r="C19" s="9" t="s">
+      <c r="C19" t="s">
         <v>182</v>
       </c>
       <c r="D19">
@@ -3128,7 +3151,7 @@
         <v>160</v>
       </c>
       <c r="L19" t="s">
-        <v>194</v>
+        <v>323</v>
       </c>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.25">
@@ -3138,7 +3161,7 @@
       <c r="B20" t="s">
         <v>179</v>
       </c>
-      <c r="C20" s="9">
+      <c r="C20">
         <v>2025</v>
       </c>
       <c r="D20">
@@ -3157,7 +3180,7 @@
         <v>160</v>
       </c>
       <c r="L20" t="s">
-        <v>193</v>
+        <v>322</v>
       </c>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.25">
@@ -3167,7 +3190,7 @@
       <c r="B21" t="s">
         <v>180</v>
       </c>
-      <c r="C21" s="9">
+      <c r="C21">
         <v>2025</v>
       </c>
       <c r="D21">
@@ -3186,7 +3209,7 @@
         <v>160</v>
       </c>
       <c r="L21" t="s">
-        <v>193</v>
+        <v>322</v>
       </c>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.25">
@@ -3196,7 +3219,7 @@
       <c r="B22" t="s">
         <v>155</v>
       </c>
-      <c r="C22" s="9" t="s">
+      <c r="C22" t="s">
         <v>171</v>
       </c>
       <c r="D22">
@@ -3231,7 +3254,7 @@
       <c r="B23" t="s">
         <v>31</v>
       </c>
-      <c r="C23" s="9" t="s">
+      <c r="C23" t="s">
         <v>184</v>
       </c>
       <c r="D23">
@@ -3266,7 +3289,7 @@
       <c r="B24" t="s">
         <v>175</v>
       </c>
-      <c r="C24" s="9">
+      <c r="C24">
         <v>2019</v>
       </c>
       <c r="D24">
@@ -3285,7 +3308,7 @@
         <v>160</v>
       </c>
       <c r="L24" t="s">
-        <v>193</v>
+        <v>322</v>
       </c>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.25">
@@ -3295,7 +3318,7 @@
       <c r="B25" t="s">
         <v>9</v>
       </c>
-      <c r="C25" s="9" t="s">
+      <c r="C25" t="s">
         <v>173</v>
       </c>
       <c r="D25">
@@ -3330,7 +3353,7 @@
       <c r="B26" t="s">
         <v>164</v>
       </c>
-      <c r="C26" s="9" t="s">
+      <c r="C26" t="s">
         <v>173</v>
       </c>
       <c r="D26">
@@ -3365,7 +3388,7 @@
       <c r="B27" t="s">
         <v>162</v>
       </c>
-      <c r="C27" s="9" t="s">
+      <c r="C27" t="s">
         <v>172</v>
       </c>
       <c r="D27">
@@ -3388,6 +3411,9 @@
       </c>
       <c r="K27" t="s">
         <v>160</v>
+      </c>
+      <c r="L27" t="s">
+        <v>325</v>
       </c>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.25">
@@ -3397,7 +3423,7 @@
       <c r="B28" t="s">
         <v>33</v>
       </c>
-      <c r="C28" s="9" t="s">
+      <c r="C28" t="s">
         <v>171</v>
       </c>
       <c r="D28">
@@ -3432,7 +3458,7 @@
       <c r="B29" t="s">
         <v>174</v>
       </c>
-      <c r="C29" s="9">
+      <c r="C29">
         <v>2018</v>
       </c>
       <c r="D29">
@@ -3451,7 +3477,7 @@
         <v>160</v>
       </c>
       <c r="L29" t="s">
-        <v>193</v>
+        <v>322</v>
       </c>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.25">
@@ -3461,7 +3487,7 @@
       <c r="B30" t="s">
         <v>161</v>
       </c>
-      <c r="C30" s="9" t="s">
+      <c r="C30" t="s">
         <v>182</v>
       </c>
       <c r="D30">
@@ -3486,7 +3512,7 @@
         <v>160</v>
       </c>
       <c r="L30" t="s">
-        <v>194</v>
+        <v>323</v>
       </c>
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.25">
@@ -3496,7 +3522,7 @@
       <c r="B31" t="s">
         <v>169</v>
       </c>
-      <c r="C31" s="9" t="s">
+      <c r="C31" t="s">
         <v>185</v>
       </c>
       <c r="D31">
@@ -3521,7 +3547,7 @@
         <v>160</v>
       </c>
       <c r="L31" t="s">
-        <v>194</v>
+        <v>323</v>
       </c>
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.25">
@@ -3531,7 +3557,7 @@
       <c r="B32" t="s">
         <v>37</v>
       </c>
-      <c r="C32" s="9" t="s">
+      <c r="C32" t="s">
         <v>171</v>
       </c>
       <c r="D32">
@@ -3549,15 +3575,18 @@
       <c r="K32" t="s">
         <v>160</v>
       </c>
+      <c r="L32" t="s">
+        <v>324</v>
+      </c>
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B33" t="s">
         <v>163</v>
       </c>
-      <c r="C33" s="9" t="s">
+      <c r="C33" t="s">
         <v>171</v>
       </c>
       <c r="D33">
@@ -3600,7 +3629,7 @@
     <col min="2" max="2" width="29.140625" customWidth="1"/>
     <col min="3" max="3" width="10.7109375" customWidth="1"/>
     <col min="4" max="4" width="10.42578125" customWidth="1"/>
-    <col min="5" max="5" width="12" customWidth="1"/>
+    <col min="5" max="5" width="80.7109375" customWidth="1"/>
     <col min="6" max="6" width="28.7109375" customWidth="1"/>
     <col min="7" max="7" width="28.42578125" customWidth="1"/>
     <col min="8" max="8" width="13.85546875" customWidth="1"/>
@@ -4242,7 +4271,7 @@
       <c r="D14">
         <v>93544</v>
       </c>
-      <c r="E14" s="5" t="s">
+      <c r="E14" s="9" t="s">
         <v>129</v>
       </c>
       <c r="F14" s="6">
@@ -4712,7 +4741,7 @@
       <c r="D24">
         <v>188448</v>
       </c>
-      <c r="E24" s="5" t="s">
+      <c r="E24" s="9" t="s">
         <v>139</v>
       </c>
       <c r="F24" s="6">
@@ -5041,7 +5070,7 @@
       <c r="D31">
         <v>188347</v>
       </c>
-      <c r="E31" s="5" t="s">
+      <c r="E31" s="9" t="s">
         <v>146</v>
       </c>
       <c r="F31" s="6">
@@ -5350,4 +5379,10 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{490a8197-7b83-4f10-89b9-83189be3835e}" enabled="0" method="" siteId="{490a8197-7b83-4f10-89b9-83189be3835e}" removed="1"/>
+</clbl:labelList>
 </file>
</xml_diff>

<commit_message>
Update CNC metadata workbook
</commit_message>
<xml_diff>
--- a/CNC_UK_data_overview.xlsx
+++ b/CNC_UK_data_overview.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hullacuk-my.sharepoint.com/personal/b_hodgson-2022_hull_ac_uk/Documents/Aa. Dissertation/Data and Analysis/GitHub folder/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="401" documentId="11_40EA3C77D094CE56413DCE42115AF69F046E0E85" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2D79F7A7-4A78-48D8-9342-68C5DD9DF06F}"/>
+  <xr:revisionPtr revIDLastSave="407" documentId="11_40EA3C77D094CE56413DCE42115AF69F046E0E85" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E9682236-8887-44DB-BA8B-3620007B208C}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Participation_by_year" sheetId="5" r:id="rId1"/>
@@ -3566,6 +3566,9 @@
       <c r="E32">
         <v>3</v>
       </c>
+      <c r="G32">
+        <v>10</v>
+      </c>
       <c r="H32">
         <v>51.62</v>
       </c>
@@ -3576,7 +3579,7 @@
         <v>160</v>
       </c>
       <c r="L32" t="s">
-        <v>324</v>
+        <v>192</v>
       </c>
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.25">

</xml_diff>